<commit_message>
Add Playwright login tests with screenshots embedded in Excel
test/test_login.py: 13件の自動テスト（成功3件・失敗10件）
test/screenshots/: 各テストのスクリーンショット（PNG）
ログインテスト仕様書.xlsx: 各明細Noシートにスクリーンショット貼付
requirements.txt: openpyxl / Pillow / playwright を追加

Co-Authored-By: Claude Sonnet 4.6 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/test/ログインテスト仕様書.xlsx
+++ b/test/ログインテスト仕様書.xlsx
@@ -242,6 +242,396 @@
     </indexedColors>
   </colors>
 </styleSheet>
+</file>
+
+<file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing10.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing11.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing12.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing13.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing2.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing4.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing5.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing6.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing7.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing8.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing9.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>2</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="8572500" cy="5362575"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId1"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -1121,11 +1511,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1148,11 +1540,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1175,11 +1569,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1202,11 +1598,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1229,11 +1627,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1256,11 +1656,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1283,11 +1685,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1310,11 +1714,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1337,11 +1743,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1364,11 +1772,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1391,11 +1801,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1418,11 +1830,13 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
 
@@ -1445,10 +1859,12 @@
         </is>
       </c>
     </row>
+    <row r="3" ht="430" customHeight="1"/>
   </sheetData>
   <mergeCells count="1">
     <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
 </worksheet>
 </file>
</xml_diff>